<commit_message>
Works with bugs, Need to find a more elegant solution to enlarge / detract cards, advance turns etc but play mostly works
</commit_message>
<xml_diff>
--- a/CardGameInterface.xlsx
+++ b/CardGameInterface.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Benjamin Ellinger\Desktop\Digipen\DES315\Grading\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gary Yang\Documents\Programing\Unity\CardStuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB39F55-D930-4BA2-B15B-C4DCE9A0A73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFD21E6-D4B8-4818-886C-87370FC70073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="66015" yWindow="2685" windowWidth="20385" windowHeight="13230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="22" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="40">
   <si>
     <t>POST-MORTEM (200+ Words)</t>
   </si>
@@ -1211,6 +1211,12 @@
       </rPr>
       <t xml:space="preserve"> if well-crafted with sophisticated animations when going both in and out.</t>
     </r>
+  </si>
+  <si>
+    <t>Full Credit</t>
+  </si>
+  <si>
+    <t>Partial Credit</t>
   </si>
 </sst>
 </file>
@@ -1671,60 +1677,32 @@
   </cellStyles>
   <dxfs count="72">
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <strike val="0"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
@@ -1740,40 +1718,54 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <strike val="0"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1790,7 +1782,28 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B0F0"/>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1800,14 +1813,35 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1824,6 +1858,48 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="9"/>
         </patternFill>
       </fill>
@@ -1832,34 +1908,6 @@
       <fill>
         <patternFill>
           <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1869,41 +1917,6 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="9"/>
         </patternFill>
       </fill>
@@ -1921,7 +1934,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
+          <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1945,13 +1958,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
@@ -2045,7 +2051,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2091,6 +2104,13 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <strike val="0"/>
       </font>
@@ -2110,13 +2130,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
@@ -2131,7 +2144,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B0F0"/>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2141,28 +2168,14 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2172,7 +2185,21 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2186,21 +2213,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
+          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2208,13 +2221,6 @@
       <font>
         <strike val="0"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="7" tint="0.39994506668294322"/>
@@ -2518,7 +2524,7 @@
     <row r="1" spans="1:5" s="3" customFormat="1" ht="23.4" thickBot="1">
       <c r="A1" s="18">
         <f>MIN(1,(MAX(D1,(SUM(A4:A963)+IF(ISBLANK(A2),0,MIN(0,A2-0.7))))))</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="B1" s="32" t="s">
         <v>8</v>
@@ -2528,7 +2534,7 @@
       </c>
       <c r="D1" s="33">
         <f>MAX(A6,0)+MAX(A11,0)+MAX(A16,0)+MAX(A21,0)+MAX(A26,0)+MAX(A31,0)+COUNTIF(A7:A9,"&gt;0")*0.01+COUNTIF(A12:A14,"&gt;0")*0.01+COUNTIF(A17:A19,"&gt;0")*0.01+COUNTIF(A22:A24,"&gt;0")*0.01+COUNTIF(A27:A28,"&gt;0")*0.01+COUNTIF(A32:A34,"&gt;0")*0.01</f>
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="E1" s="9"/>
     </row>
@@ -2574,33 +2580,39 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A7" s="34" t="str">
+      <c r="A7" s="34">
         <f>IF(LEFT(B7,2)="No",-0.1,IF(LEFT(B7,7)="Partial",0.01,IF(LEFT(B7,4)="Full",0.03,IF(LEFT(B7,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B7" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C7" s="37" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="12"/>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A8" s="34" t="str">
+      <c r="A8" s="34">
         <f>IF(LEFT(B8,2)="No",-0.1,IF(LEFT(B8,7)="Partial",0.01,IF(LEFT(B8,4)="Full",0.03,IF(LEFT(B8,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B8" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C8" s="37" t="s">
         <v>18</v>
       </c>
       <c r="E8" s="12"/>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A9" s="34" t="str">
+      <c r="A9" s="34">
         <f>IF(LEFT(B9,2)="No",-0.1,IF(LEFT(B9,7)="Partial",0.01,IF(LEFT(B9,4)="Full",0.03,IF(LEFT(B9,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B9" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C9" s="37" t="s">
         <v>20</v>
       </c>
@@ -2621,33 +2633,39 @@
       <c r="E11" s="12"/>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" ht="31.9" customHeight="1" thickBot="1">
-      <c r="A12" s="34" t="str">
+      <c r="A12" s="34">
         <f>IF(LEFT(B12,2)="No",-0.1,IF(LEFT(B12,7)="Partial",0.01,IF(LEFT(B12,4)="Full",0.03,IF(LEFT(B12,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B12" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C12" s="37" t="s">
         <v>21</v>
       </c>
       <c r="E12" s="12"/>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A13" s="34" t="str">
+      <c r="A13" s="34">
         <f>IF(LEFT(B13,2)="No",-0.1,IF(LEFT(B13,7)="Partial",0.01,IF(LEFT(B13,4)="Full",0.03,IF(LEFT(B13,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B13" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C13" s="37" t="s">
         <v>22</v>
       </c>
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A14" s="34" t="str">
+      <c r="A14" s="34">
         <f>IF(LEFT(B14,2)="No",-0.1,IF(LEFT(B14,7)="Partial",0.01,IF(LEFT(B14,4)="Full",0.03,IF(LEFT(B14,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B14" s="35"/>
+        <v>0.01</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>39</v>
+      </c>
       <c r="C14" s="37" t="s">
         <v>23</v>
       </c>
@@ -2668,33 +2686,39 @@
       <c r="E16" s="12"/>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A17" s="34" t="str">
+      <c r="A17" s="34">
         <f>IF(LEFT(B17,2)="No",-0.1,IF(LEFT(B17,7)="Partial",0.01,IF(LEFT(B17,4)="Full",0.03,IF(LEFT(B17,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B17" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C17" s="37" t="s">
         <v>24</v>
       </c>
       <c r="E17" s="12"/>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" ht="31.9" customHeight="1" thickBot="1">
-      <c r="A18" s="34" t="str">
+      <c r="A18" s="34">
         <f>IF(LEFT(B18,2)="No",-0.1,IF(LEFT(B18,7)="Partial",0.01,IF(LEFT(B18,4)="Full",0.03,IF(LEFT(B18,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B18" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C18" s="37" t="s">
         <v>25</v>
       </c>
       <c r="E18" s="11"/>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" ht="31.5" thickBot="1">
-      <c r="A19" s="34" t="str">
+      <c r="A19" s="34">
         <f>IF(LEFT(B19,2)="No",-0.1,IF(LEFT(B19,7)="Partial",0.01,IF(LEFT(B19,4)="Full",0.03,IF(LEFT(B19,5)="Extra",0.05,"n/a"))))</f>
-        <v>n/a</v>
-      </c>
-      <c r="B19" s="35"/>
+        <v>0.03</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="C19" s="37" t="s">
         <v>28</v>
       </c>
@@ -2908,76 +2932,76 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B9">
-    <cfRule type="beginsWith" dxfId="70" priority="90" stopIfTrue="1" operator="beginsWith" text="Small">
+    <cfRule type="beginsWith" dxfId="70" priority="89" stopIfTrue="1" operator="beginsWith" text="No Progress">
+      <formula>LEFT(B6,LEN("No Progress"))="No Progress"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="69" priority="98" stopIfTrue="1" operator="beginsWith" text="Lots">
+      <formula>LEFT(B6,LEN("Lots"))="Lots"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="68" priority="94" stopIfTrue="1" operator="endsWith" text="Met">
+      <formula>RIGHT(B6,LEN("Met"))="Met"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="67" priority="93" stopIfTrue="1" operator="beginsWith" text="Big">
+      <formula>LEFT(B6,LEN("Big"))="Big"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="66" priority="92" stopIfTrue="1" operator="beginsWith" text="Full">
+      <formula>LEFT(B6,LEN("Full"))="Full"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="65" priority="91" stopIfTrue="1" operator="beginsWith" text="Some">
+      <formula>LEFT(B6,LEN("Some"))="Some"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="64" priority="90" stopIfTrue="1" operator="beginsWith" text="Small">
       <formula>LEFT(B6,LEN("Small"))="Small"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="69" priority="89" stopIfTrue="1" operator="beginsWith" text="No Progress">
-      <formula>LEFT(B6,LEN("No Progress"))="No Progress"</formula>
-    </cfRule>
-    <cfRule type="endsWith" dxfId="68" priority="87" stopIfTrue="1" operator="endsWith" text="Missed">
+    <cfRule type="beginsWith" dxfId="63" priority="88" stopIfTrue="1" operator="beginsWith" text="Partial">
+      <formula>LEFT(B6,LEN("Partial"))="Partial"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="62" priority="87" stopIfTrue="1" operator="endsWith" text="Missed">
       <formula>RIGHT(B6,LEN("Missed"))="Missed"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="67" priority="86" stopIfTrue="1" operator="beginsWith" text="Not">
+    <cfRule type="beginsWith" dxfId="61" priority="86" stopIfTrue="1" operator="beginsWith" text="Not">
       <formula>LEFT(B6,LEN("Not"))="Not"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="66" priority="85" stopIfTrue="1" operator="beginsWith" text="No Credit">
+    <cfRule type="beginsWith" dxfId="60" priority="85" stopIfTrue="1" operator="beginsWith" text="No Credit">
       <formula>LEFT(B6,LEN("No Credit"))="No Credit"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="65" priority="98" stopIfTrue="1" operator="beginsWith" text="Lots">
-      <formula>LEFT(B6,LEN("Lots"))="Lots"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="64" priority="88" stopIfTrue="1" operator="beginsWith" text="Partial">
-      <formula>LEFT(B6,LEN("Partial"))="Partial"</formula>
-    </cfRule>
-    <cfRule type="endsWith" dxfId="63" priority="94" stopIfTrue="1" operator="endsWith" text="Met">
-      <formula>RIGHT(B6,LEN("Met"))="Met"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="62" priority="93" stopIfTrue="1" operator="beginsWith" text="Big">
-      <formula>LEFT(B6,LEN("Big"))="Big"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="61" priority="92" stopIfTrue="1" operator="beginsWith" text="Full">
-      <formula>LEFT(B6,LEN("Full"))="Full"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="60" priority="91" stopIfTrue="1" operator="beginsWith" text="Some">
-      <formula>LEFT(B6,LEN("Some"))="Some"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:B14 B26:B29">
-    <cfRule type="beginsWith" dxfId="59" priority="84" stopIfTrue="1" operator="beginsWith" text="Lots">
+    <cfRule type="beginsWith" dxfId="59" priority="83" stopIfTrue="1" operator="beginsWith" text="Extra">
+      <formula>LEFT(B11,LEN("Extra"))="Extra"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="58" priority="82" stopIfTrue="1" operator="endsWith" text="Met">
+      <formula>RIGHT(B11,LEN("Met"))="Met"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="57" priority="81" stopIfTrue="1" operator="beginsWith" text="Big">
+      <formula>LEFT(B11,LEN("Big"))="Big"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="56" priority="79" stopIfTrue="1" operator="beginsWith" text="Some">
+      <formula>LEFT(B11,LEN("Some"))="Some"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="55" priority="78" stopIfTrue="1" operator="beginsWith" text="Small">
+      <formula>LEFT(B11,LEN("Small"))="Small"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="54" priority="77" stopIfTrue="1" operator="beginsWith" text="No Progress">
+      <formula>LEFT(B11,LEN("No Progress"))="No Progress"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="53" priority="76" stopIfTrue="1" operator="beginsWith" text="Partial">
+      <formula>LEFT(B11,LEN("Partial"))="Partial"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="52" priority="75" stopIfTrue="1" operator="endsWith" text="Missed">
+      <formula>RIGHT(B11,LEN("Missed"))="Missed"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="51" priority="74" stopIfTrue="1" operator="beginsWith" text="Not">
+      <formula>LEFT(B11,LEN("Not"))="Not"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="50" priority="73" stopIfTrue="1" operator="beginsWith" text="No Credit">
+      <formula>LEFT(B11,LEN("No Credit"))="No Credit"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="49" priority="80" stopIfTrue="1" operator="beginsWith" text="Full">
+      <formula>LEFT(B11,LEN("Full"))="Full"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="48" priority="84" stopIfTrue="1" operator="beginsWith" text="Lots">
       <formula>LEFT(B11,LEN("Lots"))="Lots"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="58" priority="83" stopIfTrue="1" operator="beginsWith" text="Extra">
-      <formula>LEFT(B11,LEN("Extra"))="Extra"</formula>
-    </cfRule>
-    <cfRule type="endsWith" dxfId="57" priority="82" stopIfTrue="1" operator="endsWith" text="Met">
-      <formula>RIGHT(B11,LEN("Met"))="Met"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="56" priority="81" stopIfTrue="1" operator="beginsWith" text="Big">
-      <formula>LEFT(B11,LEN("Big"))="Big"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="55" priority="80" stopIfTrue="1" operator="beginsWith" text="Full">
-      <formula>LEFT(B11,LEN("Full"))="Full"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="54" priority="79" stopIfTrue="1" operator="beginsWith" text="Some">
-      <formula>LEFT(B11,LEN("Some"))="Some"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="53" priority="77" stopIfTrue="1" operator="beginsWith" text="No Progress">
-      <formula>LEFT(B11,LEN("No Progress"))="No Progress"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="52" priority="76" stopIfTrue="1" operator="beginsWith" text="Partial">
-      <formula>LEFT(B11,LEN("Partial"))="Partial"</formula>
-    </cfRule>
-    <cfRule type="endsWith" dxfId="51" priority="75" stopIfTrue="1" operator="endsWith" text="Missed">
-      <formula>RIGHT(B11,LEN("Missed"))="Missed"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="50" priority="74" stopIfTrue="1" operator="beginsWith" text="Not">
-      <formula>LEFT(B11,LEN("Not"))="Not"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="49" priority="73" stopIfTrue="1" operator="beginsWith" text="No Credit">
-      <formula>LEFT(B11,LEN("No Credit"))="No Credit"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="48" priority="78" stopIfTrue="1" operator="beginsWith" text="Small">
-      <formula>LEFT(B11,LEN("Small"))="Small"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:B19">
@@ -3008,128 +3032,128 @@
     <cfRule type="beginsWith" dxfId="39" priority="9" stopIfTrue="1" operator="beginsWith" text="Big">
       <formula>LEFT(B16,LEN("Big"))="Big"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="38" priority="10" stopIfTrue="1" operator="endsWith" text="Met">
-      <formula>RIGHT(B16,LEN("Met"))="Met"</formula>
+    <cfRule type="beginsWith" dxfId="38" priority="11" stopIfTrue="1" operator="beginsWith" text="Extra">
+      <formula>LEFT(B16,LEN("Extra"))="Extra"</formula>
     </cfRule>
     <cfRule type="beginsWith" dxfId="37" priority="12" stopIfTrue="1" operator="beginsWith" text="Lots">
       <formula>LEFT(B16,LEN("Lots"))="Lots"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="36" priority="11" stopIfTrue="1" operator="beginsWith" text="Extra">
-      <formula>LEFT(B16,LEN("Extra"))="Extra"</formula>
+    <cfRule type="endsWith" dxfId="36" priority="10" stopIfTrue="1" operator="endsWith" text="Met">
+      <formula>RIGHT(B16,LEN("Met"))="Met"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:B24">
-    <cfRule type="beginsWith" dxfId="35" priority="57" stopIfTrue="1" operator="beginsWith" text="Big">
-      <formula>LEFT(B21,LEN("Big"))="Big"</formula>
-    </cfRule>
-    <cfRule type="endsWith" dxfId="34" priority="51" stopIfTrue="1" operator="endsWith" text="Missed">
+    <cfRule type="endsWith" dxfId="35" priority="51" stopIfTrue="1" operator="endsWith" text="Missed">
       <formula>RIGHT(B21,LEN("Missed"))="Missed"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="33" priority="52" stopIfTrue="1" operator="beginsWith" text="Partial">
+    <cfRule type="beginsWith" dxfId="34" priority="52" stopIfTrue="1" operator="beginsWith" text="Partial">
       <formula>LEFT(B21,LEN("Partial"))="Partial"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="32" priority="55" stopIfTrue="1" operator="beginsWith" text="Some">
+    <cfRule type="beginsWith" dxfId="33" priority="53" stopIfTrue="1" operator="beginsWith" text="No Progress">
+      <formula>LEFT(B21,LEN("No Progress"))="No Progress"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="32" priority="54" stopIfTrue="1" operator="beginsWith" text="Small">
+      <formula>LEFT(B21,LEN("Small"))="Small"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="31" priority="55" stopIfTrue="1" operator="beginsWith" text="Some">
       <formula>LEFT(B21,LEN("Some"))="Some"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="31" priority="54" stopIfTrue="1" operator="beginsWith" text="Small">
-      <formula>LEFT(B21,LEN("Small"))="Small"</formula>
     </cfRule>
     <cfRule type="beginsWith" dxfId="30" priority="56" stopIfTrue="1" operator="beginsWith" text="Full">
       <formula>LEFT(B21,LEN("Full"))="Full"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="29" priority="49" stopIfTrue="1" operator="beginsWith" text="No Credit">
-      <formula>LEFT(B21,LEN("No Credit"))="No Credit"</formula>
+    <cfRule type="beginsWith" dxfId="29" priority="57" stopIfTrue="1" operator="beginsWith" text="Big">
+      <formula>LEFT(B21,LEN("Big"))="Big"</formula>
     </cfRule>
     <cfRule type="endsWith" dxfId="28" priority="58" stopIfTrue="1" operator="endsWith" text="Met">
       <formula>RIGHT(B21,LEN("Met"))="Met"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="27" priority="59" stopIfTrue="1" operator="beginsWith" text="Extra">
-      <formula>LEFT(B21,LEN("Extra"))="Extra"</formula>
+    <cfRule type="beginsWith" dxfId="27" priority="50" stopIfTrue="1" operator="beginsWith" text="Not">
+      <formula>LEFT(B21,LEN("Not"))="Not"</formula>
     </cfRule>
     <cfRule type="beginsWith" dxfId="26" priority="60" stopIfTrue="1" operator="beginsWith" text="Lots">
       <formula>LEFT(B21,LEN("Lots"))="Lots"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="25" priority="53" stopIfTrue="1" operator="beginsWith" text="No Progress">
-      <formula>LEFT(B21,LEN("No Progress"))="No Progress"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="24" priority="50" stopIfTrue="1" operator="beginsWith" text="Not">
-      <formula>LEFT(B21,LEN("Not"))="Not"</formula>
+    <cfRule type="beginsWith" dxfId="25" priority="49" stopIfTrue="1" operator="beginsWith" text="No Credit">
+      <formula>LEFT(B21,LEN("No Credit"))="No Credit"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="24" priority="59" stopIfTrue="1" operator="beginsWith" text="Extra">
+      <formula>LEFT(B21,LEN("Extra"))="Extra"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31:B34">
-    <cfRule type="beginsWith" dxfId="23" priority="25" stopIfTrue="1" operator="beginsWith" text="No Credit">
-      <formula>LEFT(B31,LEN("No Credit"))="No Credit"</formula>
+    <cfRule type="beginsWith" dxfId="23" priority="29" stopIfTrue="1" operator="beginsWith" text="No Progress">
+      <formula>LEFT(B31,LEN("No Progress"))="No Progress"</formula>
     </cfRule>
     <cfRule type="beginsWith" dxfId="22" priority="36" stopIfTrue="1" operator="beginsWith" text="Lots">
       <formula>LEFT(B31,LEN("Lots"))="Lots"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="21" priority="33" stopIfTrue="1" operator="beginsWith" text="Big">
+    <cfRule type="beginsWith" dxfId="21" priority="35" stopIfTrue="1" operator="beginsWith" text="Extra">
+      <formula>LEFT(B31,LEN("Extra"))="Extra"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="20" priority="34" stopIfTrue="1" operator="endsWith" text="Met">
+      <formula>RIGHT(B31,LEN("Met"))="Met"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="19" priority="33" stopIfTrue="1" operator="beginsWith" text="Big">
       <formula>LEFT(B31,LEN("Big"))="Big"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="20" priority="32" stopIfTrue="1" operator="beginsWith" text="Full">
+    <cfRule type="beginsWith" dxfId="18" priority="32" stopIfTrue="1" operator="beginsWith" text="Full">
       <formula>LEFT(B31,LEN("Full"))="Full"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="19" priority="31" stopIfTrue="1" operator="beginsWith" text="Some">
+    <cfRule type="beginsWith" dxfId="17" priority="31" stopIfTrue="1" operator="beginsWith" text="Some">
       <formula>LEFT(B31,LEN("Some"))="Some"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="18" priority="35" stopIfTrue="1" operator="beginsWith" text="Extra">
-      <formula>LEFT(B31,LEN("Extra"))="Extra"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="17" priority="30" stopIfTrue="1" operator="beginsWith" text="Small">
+    <cfRule type="beginsWith" dxfId="16" priority="30" stopIfTrue="1" operator="beginsWith" text="Small">
       <formula>LEFT(B31,LEN("Small"))="Small"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="16" priority="29" stopIfTrue="1" operator="beginsWith" text="No Progress">
-      <formula>LEFT(B31,LEN("No Progress"))="No Progress"</formula>
-    </cfRule>
-    <cfRule type="endsWith" dxfId="15" priority="34" stopIfTrue="1" operator="endsWith" text="Met">
-      <formula>RIGHT(B31,LEN("Met"))="Met"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="14" priority="28" stopIfTrue="1" operator="beginsWith" text="Partial">
+    <cfRule type="endsWith" dxfId="15" priority="27" stopIfTrue="1" operator="endsWith" text="Missed">
+      <formula>RIGHT(B31,LEN("Missed"))="Missed"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="14" priority="26" stopIfTrue="1" operator="beginsWith" text="Not">
+      <formula>LEFT(B31,LEN("Not"))="Not"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="13" priority="25" stopIfTrue="1" operator="beginsWith" text="No Credit">
+      <formula>LEFT(B31,LEN("No Credit"))="No Credit"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="12" priority="28" stopIfTrue="1" operator="beginsWith" text="Partial">
       <formula>LEFT(B31,LEN("Partial"))="Partial"</formula>
-    </cfRule>
-    <cfRule type="endsWith" dxfId="13" priority="27" stopIfTrue="1" operator="endsWith" text="Missed">
-      <formula>RIGHT(B31,LEN("Missed"))="Missed"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="12" priority="26" stopIfTrue="1" operator="beginsWith" text="Not">
-      <formula>LEFT(B31,LEN("Not"))="Not"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B36">
-    <cfRule type="beginsWith" dxfId="11" priority="14" stopIfTrue="1" operator="beginsWith" text="Not">
+    <cfRule type="beginsWith" dxfId="11" priority="24" stopIfTrue="1" operator="beginsWith" text="Lots">
+      <formula>LEFT(B36,LEN("Lots"))="Lots"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="10" priority="23" stopIfTrue="1" operator="beginsWith" text="Extra">
+      <formula>LEFT(B36,LEN("Extra"))="Extra"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="9" priority="22" stopIfTrue="1" operator="endsWith" text="Met">
+      <formula>RIGHT(B36,LEN("Met"))="Met"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="8" priority="21" stopIfTrue="1" operator="beginsWith" text="Big">
+      <formula>LEFT(B36,LEN("Big"))="Big"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="7" priority="20" stopIfTrue="1" operator="beginsWith" text="Full">
+      <formula>LEFT(B36,LEN("Full"))="Full"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="6" priority="19" stopIfTrue="1" operator="beginsWith" text="Some">
+      <formula>LEFT(B36,LEN("Some"))="Some"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="5" priority="18" stopIfTrue="1" operator="beginsWith" text="Small">
+      <formula>LEFT(B36,LEN("Small"))="Small"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="4" priority="17" stopIfTrue="1" operator="beginsWith" text="No Progress">
+      <formula>LEFT(B36,LEN("No Progress"))="No Progress"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="3" priority="16" stopIfTrue="1" operator="beginsWith" text="Partial">
+      <formula>LEFT(B36,LEN("Partial"))="Partial"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="2" priority="15" stopIfTrue="1" operator="endsWith" text="Missed">
+      <formula>RIGHT(B36,LEN("Missed"))="Missed"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="1" priority="14" stopIfTrue="1" operator="beginsWith" text="Not">
       <formula>LEFT(B36,LEN("Not"))="Not"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="10" priority="15" stopIfTrue="1" operator="endsWith" text="Missed">
-      <formula>RIGHT(B36,LEN("Missed"))="Missed"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="9" priority="16" stopIfTrue="1" operator="beginsWith" text="Partial">
-      <formula>LEFT(B36,LEN("Partial"))="Partial"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="8" priority="17" stopIfTrue="1" operator="beginsWith" text="No Progress">
-      <formula>LEFT(B36,LEN("No Progress"))="No Progress"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="7" priority="18" stopIfTrue="1" operator="beginsWith" text="Small">
-      <formula>LEFT(B36,LEN("Small"))="Small"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="6" priority="13" stopIfTrue="1" operator="beginsWith" text="No Credit">
+    <cfRule type="beginsWith" dxfId="0" priority="13" stopIfTrue="1" operator="beginsWith" text="No Credit">
       <formula>LEFT(B36,LEN("No Credit"))="No Credit"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="5" priority="24" stopIfTrue="1" operator="beginsWith" text="Lots">
-      <formula>LEFT(B36,LEN("Lots"))="Lots"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="4" priority="23" stopIfTrue="1" operator="beginsWith" text="Extra">
-      <formula>LEFT(B36,LEN("Extra"))="Extra"</formula>
-    </cfRule>
-    <cfRule type="endsWith" dxfId="3" priority="22" stopIfTrue="1" operator="endsWith" text="Met">
-      <formula>RIGHT(B36,LEN("Met"))="Met"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="2" priority="21" stopIfTrue="1" operator="beginsWith" text="Big">
-      <formula>LEFT(B36,LEN("Big"))="Big"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="1" priority="20" stopIfTrue="1" operator="beginsWith" text="Full">
-      <formula>LEFT(B36,LEN("Full"))="Full"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="0" priority="19" stopIfTrue="1" operator="beginsWith" text="Some">
-      <formula>LEFT(B36,LEN("Some"))="Some"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">

</xml_diff>

<commit_message>
added telemetry class, moslty feature complete game wise
</commit_message>
<xml_diff>
--- a/CardGameInterface.xlsx
+++ b/CardGameInterface.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gary Yang\Documents\Programing\Unity\CardStuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFD21E6-D4B8-4818-886C-87370FC70073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50FA55D5-292F-4620-9083-DF43A3D01B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <sheet name="Code Report" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>